<commit_message>
PATCH-11: Enhance logging, report and customize selenium grid command
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/leapfrog/leapfrog-games.xlsx
+++ b/src/test/resources/testdata/leapfrog/leapfrog-games.xlsx
@@ -2830,7 +2830,7 @@
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -4351,16 +4351,16 @@
       <c r="B141" t="s">
         <v>160</v>
       </c>
-      <c r="C141" t="s">
-        <v>5</v>
+      <c r="C141" s="1" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="s">
         <v>161</v>
       </c>
-      <c r="B142" t="s">
-        <v>7</v>
+      <c r="B142" s="1" t="s">
+        <v>160</v>
       </c>
       <c r="C142" t="s">
         <v>5</v>
@@ -6900,11 +6900,11 @@
       <c r="A373" t="s">
         <v>398</v>
       </c>
-      <c r="B373" t="s">
-        <v>22</v>
-      </c>
-      <c r="C373" t="s">
-        <v>5</v>
+      <c r="B373" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C373" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="374">
@@ -7750,8 +7750,8 @@
       <c r="B450" t="s">
         <v>24</v>
       </c>
-      <c r="C450" t="s">
-        <v>13</v>
+      <c r="C450" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="451">
@@ -10135,7 +10135,7 @@
         <v>692</v>
       </c>
       <c r="B667" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C667" t="s">
         <v>13</v>

</xml_diff>